<commit_message>
add remark at the bottom of the output
</commit_message>
<xml_diff>
--- a/ตัวอย่างใบสั่งซื้อต่างประเทศ.xlsx
+++ b/ตัวอย่างใบสั่งซื้อต่างประเทศ.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10222"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PO\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/KUNTIDA/PO/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86F90D1F-D30A-45D2-A972-D4B90756C01C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F88F294-3EC2-0D48-9A17-E2A882E53BD4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{236A65F7-5668-4671-A38E-59B8E218F7F2}"/>
+    <workbookView xWindow="6980" yWindow="3420" windowWidth="23260" windowHeight="13900" xr2:uid="{236A65F7-5668-4671-A38E-59B8E218F7F2}"/>
   </bookViews>
   <sheets>
     <sheet name="page1" sheetId="6" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="37">
   <si>
     <t>GREENLIFE ENTERPRISES CO., LTD.</t>
   </si>
@@ -144,6 +144,12 @@
   </si>
   <si>
     <t>TOTAL QTY (ORDER)</t>
+  </si>
+  <si>
+    <t>REMARK:</t>
+  </si>
+  <si>
+    <t>เอกสารชุดนี้ได้ผ่านการตรวจสอบความถูกต้องจากผู้จัดทำแล้ว 100%</t>
   </si>
 </sst>
 </file>
@@ -151,19 +157,19 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="11">
-    <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="164" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="165" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="166" formatCode="[$-1070000]d/m/yy;@"/>
-    <numFmt numFmtId="167" formatCode="_ [$¥-804]* #,##0.000_ ;_ [$¥-804]* \-#,##0.000_ ;_ [$¥-804]* &quot;-&quot;???_ ;_ @_ "/>
-    <numFmt numFmtId="168" formatCode="_ [$¥-804]* #,##0.00_ ;_ [$¥-804]* \-#,##0.00_ ;_ [$¥-804]* &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="169" formatCode="_-[$฿-41E]* #,##0_-;\-[$฿-41E]* #,##0_-;_-[$฿-41E]* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="170" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="171" formatCode="&quot;￥&quot;#,##0.0_);[Red]\(&quot;￥&quot;#,##0.0\)"/>
-    <numFmt numFmtId="172" formatCode="[$¥-804]#,##0.00"/>
-    <numFmt numFmtId="173" formatCode="_-[$฿-41E]* #,##0.00_-;\-[$฿-41E]* #,##0.00_-;_-[$฿-41E]* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="165" formatCode="[$-1070000]d/m/yy;@"/>
+    <numFmt numFmtId="166" formatCode="_ [$¥-804]* #,##0.000_ ;_ [$¥-804]* \-#,##0.000_ ;_ [$¥-804]* &quot;-&quot;???_ ;_ @_ "/>
+    <numFmt numFmtId="167" formatCode="_ [$¥-804]* #,##0.00_ ;_ [$¥-804]* \-#,##0.00_ ;_ [$¥-804]* &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="168" formatCode="_-[$฿-41E]* #,##0_-;\-[$฿-41E]* #,##0_-;_-[$฿-41E]* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="169" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="170" formatCode="&quot;￥&quot;#,##0.0_);[Red]\(&quot;￥&quot;#,##0.0\)"/>
+    <numFmt numFmtId="171" formatCode="[$¥-804]#,##0.00"/>
+    <numFmt numFmtId="172" formatCode="_-[$฿-41E]* #,##0.00_-;\-[$฿-41E]* #,##0.00_-;_-[$฿-41E]* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="46">
+  <fonts count="47">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -192,6 +198,8 @@
       <b/>
       <sz val="24"/>
       <name val="Sukhumvit Set"/>
+      <family val="2"/>
+      <charset val="222"/>
     </font>
     <font>
       <sz val="14"/>
@@ -220,6 +228,8 @@
     <font>
       <sz val="16"/>
       <name val="Sukhumvit Set"/>
+      <family val="2"/>
+      <charset val="222"/>
     </font>
     <font>
       <sz val="18"/>
@@ -433,6 +443,11 @@
       <color indexed="8"/>
       <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="28"/>
+      <name val="Angsana New"/>
+      <family val="1"/>
     </font>
   </fonts>
   <fills count="11">
@@ -781,20 +796,20 @@
   </borders>
   <cellStyleXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="166" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="167" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="165" fontId="15" fillId="0" borderId="0"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="44" fontId="26" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="26" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="166" fontId="15" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="164" fontId="26" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="165" fontId="26" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="167" fontId="15" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="26" fillId="0" borderId="0"/>
-    <xf numFmtId="167" fontId="28" fillId="0" borderId="0">
+    <xf numFmtId="166" fontId="28" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="31" fillId="0" borderId="0"/>
+    <xf numFmtId="165" fontId="31" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="142">
+  <cellXfs count="140">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -843,7 +858,7 @@
     <xf numFmtId="49" fontId="14" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="166" fontId="18" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="18" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="49" fontId="19" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1"/>
@@ -892,10 +907,10 @@
     <xf numFmtId="0" fontId="16" fillId="2" borderId="8" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="168" fontId="16" fillId="2" borderId="7" xfId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="16" fillId="0" borderId="5" xfId="5" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="16" fillId="2" borderId="7" xfId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="168" fontId="16" fillId="0" borderId="5" xfId="5" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="1" fontId="16" fillId="3" borderId="5" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -904,13 +919,13 @@
     <xf numFmtId="1" fontId="16" fillId="5" borderId="5" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="170" fontId="16" fillId="6" borderId="5" xfId="6" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="169" fontId="16" fillId="6" borderId="5" xfId="6" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="1" fontId="16" fillId="0" borderId="5" xfId="6" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="170" fontId="25" fillId="0" borderId="5" xfId="6" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="169" fontId="25" fillId="0" borderId="5" xfId="6" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="24" fillId="0" borderId="9" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -922,7 +937,7 @@
     <xf numFmtId="49" fontId="16" fillId="2" borderId="5" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="168" fontId="16" fillId="2" borderId="11" xfId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="16" fillId="2" borderId="11" xfId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
     </xf>
     <xf numFmtId="49" fontId="27" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1"/>
@@ -945,7 +960,7 @@
     <xf numFmtId="49" fontId="16" fillId="0" borderId="5" xfId="8" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="171" fontId="16" fillId="0" borderId="5" xfId="8" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="170" fontId="16" fillId="0" borderId="5" xfId="8" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="1" fontId="16" fillId="2" borderId="5" xfId="7" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -954,10 +969,10 @@
     <xf numFmtId="3" fontId="16" fillId="3" borderId="5" xfId="7" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="170" fontId="24" fillId="6" borderId="5" xfId="6" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="169" fontId="24" fillId="6" borderId="5" xfId="6" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="29" fillId="7" borderId="0" xfId="9" applyFont="1" applyFill="1">
+    <xf numFmtId="166" fontId="29" fillId="7" borderId="0" xfId="9" applyFont="1" applyFill="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="32" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -1020,7 +1035,7 @@
     <xf numFmtId="1" fontId="25" fillId="4" borderId="10" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="168" fontId="16" fillId="0" borderId="5" xfId="6" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="16" fillId="0" borderId="5" xfId="6" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="34" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -1029,34 +1044,26 @@
     <xf numFmtId="3" fontId="35" fillId="0" borderId="5" xfId="6" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="168" fontId="37" fillId="0" borderId="4" xfId="6" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="37" fillId="0" borderId="4" xfId="6" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="168" fontId="17" fillId="2" borderId="7" xfId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="17" fillId="2" borderId="7" xfId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
     </xf>
     <xf numFmtId="49" fontId="17" fillId="2" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="49" fontId="14" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="36" fillId="2" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="39" fillId="2" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="23" fillId="2" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="49" fontId="41" fillId="2" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="1" fontId="17" fillId="4" borderId="10" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="169" fontId="5" fillId="0" borderId="5" xfId="5" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="168" fontId="5" fillId="0" borderId="5" xfId="5" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="43" fontId="43" fillId="0" borderId="12" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="43" fillId="0" borderId="12" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="173" fontId="43" fillId="8" borderId="5" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="172" fontId="43" fillId="8" borderId="5" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="49" fontId="17" fillId="0" borderId="5" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
     </xf>
@@ -1064,10 +1071,10 @@
     <xf numFmtId="49" fontId="33" fillId="0" borderId="13" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="172" fontId="16" fillId="0" borderId="7" xfId="9" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="171" fontId="16" fillId="0" borderId="7" xfId="9" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="169" fontId="16" fillId="0" borderId="9" xfId="5" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="168" fontId="16" fillId="0" borderId="9" xfId="5" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="27" fillId="0" borderId="14" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
@@ -1126,7 +1133,7 @@
     <xf numFmtId="49" fontId="16" fillId="0" borderId="5" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="45" fillId="7" borderId="5" xfId="9" applyFont="1" applyFill="1" applyBorder="1">
+    <xf numFmtId="166" fontId="45" fillId="7" borderId="5" xfId="9" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="21" fillId="9" borderId="19" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1138,6 +1145,17 @@
     <xf numFmtId="1" fontId="25" fillId="4" borderId="21" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="49" fontId="12" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="166" fontId="30" fillId="7" borderId="0" xfId="9" applyFont="1" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="46" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="49" fontId="36" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -1149,11 +1167,6 @@
     </xf>
     <xf numFmtId="49" fontId="14" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="23" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="49" fontId="12" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="167" fontId="30" fillId="7" borderId="0" xfId="9" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="11">
@@ -1187,55 +1200,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="2496207" cy="726281"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="รูปภาพ 9">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{806F20D2-C262-4F72-8136-81DF43B770ED}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill rotWithShape="1">
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:srcRect l="9014" t="25084" r="7595" b="39876"/>
-        <a:stretch/>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="2496207" cy="726281"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1539,20 +1503,20 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:BA362"/>
-  <sheetFormatPr defaultColWidth="13" defaultRowHeight="17.399999999999999"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="13" defaultRowHeight="18"/>
   <cols>
     <col min="1" max="2" width="19.6640625" style="70" customWidth="1"/>
-    <col min="3" max="3" width="34.44140625" style="74" customWidth="1"/>
-    <col min="4" max="4" width="17.5546875" style="75" customWidth="1"/>
+    <col min="3" max="3" width="34.5" style="74" customWidth="1"/>
+    <col min="4" max="4" width="17.5" style="75" customWidth="1"/>
     <col min="5" max="5" width="16" style="70" customWidth="1"/>
     <col min="6" max="6" width="14.6640625" style="75" customWidth="1"/>
     <col min="7" max="7" width="15" style="70" customWidth="1"/>
-    <col min="8" max="8" width="14.44140625" style="70" customWidth="1"/>
+    <col min="8" max="8" width="14.5" style="70" customWidth="1"/>
     <col min="9" max="10" width="16.6640625" style="76" customWidth="1"/>
     <col min="11" max="11" width="14.6640625" style="70" customWidth="1"/>
-    <col min="12" max="12" width="20.44140625" style="76" customWidth="1"/>
-    <col min="13" max="13" width="14.5546875" style="70" customWidth="1"/>
-    <col min="14" max="14" width="27.5546875" style="77" customWidth="1"/>
+    <col min="12" max="12" width="20.5" style="76" customWidth="1"/>
+    <col min="13" max="13" width="14.5" style="70" customWidth="1"/>
+    <col min="14" max="14" width="27.5" style="77" customWidth="1"/>
     <col min="15" max="16" width="14.33203125" style="78" customWidth="1"/>
     <col min="17" max="17" width="14.33203125" style="79" customWidth="1"/>
     <col min="18" max="19" width="14.33203125" style="70" customWidth="1"/>
@@ -1566,12 +1530,12 @@
     <row r="1" spans="1:53" s="3" customFormat="1" ht="36" customHeight="1">
       <c r="A1" s="1"/>
       <c r="B1" s="2"/>
-      <c r="C1" s="135" t="s">
+      <c r="C1" s="136" t="s">
         <v>0</v>
       </c>
-      <c r="D1" s="135"/>
-      <c r="E1" s="135"/>
-      <c r="F1" s="135"/>
+      <c r="D1" s="136"/>
+      <c r="E1" s="136"/>
+      <c r="F1" s="136"/>
       <c r="I1" s="4"/>
       <c r="J1" s="4"/>
       <c r="L1" s="4"/>
@@ -1632,22 +1596,22 @@
       <c r="U4" s="7"/>
     </row>
     <row r="5" spans="1:53" s="3" customFormat="1" ht="44.25" customHeight="1" thickBot="1">
-      <c r="A5" s="136" t="s">
+      <c r="A5" s="137" t="s">
         <v>1</v>
       </c>
-      <c r="B5" s="137"/>
-      <c r="C5" s="137"/>
-      <c r="D5" s="137"/>
-      <c r="E5" s="137"/>
-      <c r="F5" s="137"/>
-      <c r="G5" s="137"/>
-      <c r="H5" s="137"/>
-      <c r="I5" s="137"/>
-      <c r="J5" s="137"/>
-      <c r="K5" s="137"/>
-      <c r="L5" s="137"/>
-      <c r="M5" s="137"/>
-      <c r="N5" s="138"/>
+      <c r="B5" s="138"/>
+      <c r="C5" s="138"/>
+      <c r="D5" s="138"/>
+      <c r="E5" s="138"/>
+      <c r="F5" s="138"/>
+      <c r="G5" s="138"/>
+      <c r="H5" s="138"/>
+      <c r="I5" s="138"/>
+      <c r="J5" s="138"/>
+      <c r="K5" s="138"/>
+      <c r="L5" s="138"/>
+      <c r="M5" s="138"/>
+      <c r="N5" s="139"/>
       <c r="O5" s="97"/>
       <c r="P5" s="97"/>
       <c r="Q5" s="97"/>
@@ -1676,7 +1640,7 @@
       </c>
       <c r="N6" s="22">
         <f ca="1">NOW()</f>
-        <v>46030.720453935188</v>
+        <v>46086.567748958332</v>
       </c>
       <c r="O6" s="96"/>
       <c r="P6" s="96"/>
@@ -1736,13 +1700,13 @@
       <c r="H8" s="85" t="s">
         <v>12</v>
       </c>
-      <c r="I8" s="122" t="s">
+      <c r="I8" s="118" t="s">
         <v>6</v>
       </c>
-      <c r="J8" s="121" t="s">
+      <c r="J8" s="117" t="s">
         <v>32</v>
       </c>
-      <c r="K8" s="132" t="s">
+      <c r="K8" s="128" t="s">
         <v>34</v>
       </c>
       <c r="L8" s="83" t="s">
@@ -1763,10 +1727,10 @@
       <c r="Q8" s="31" t="s">
         <v>29</v>
       </c>
-      <c r="R8" s="123" t="s">
+      <c r="R8" s="119" t="s">
         <v>18</v>
       </c>
-      <c r="S8" s="123" t="s">
+      <c r="S8" s="119" t="s">
         <v>33</v>
       </c>
       <c r="T8" s="32" t="s">
@@ -1781,11 +1745,11 @@
       <c r="W8" s="34" t="s">
         <v>26</v>
       </c>
-      <c r="X8" s="139"/>
+      <c r="X8" s="70"/>
       <c r="Y8" s="36"/>
     </row>
-    <row r="9" spans="1:53" s="35" customFormat="1" ht="84.6" customHeight="1">
-      <c r="A9" s="106"/>
+    <row r="9" spans="1:53" s="35" customFormat="1" ht="84.5" customHeight="1">
+      <c r="A9" s="102"/>
       <c r="B9" s="88"/>
       <c r="C9" s="37"/>
       <c r="D9" s="89"/>
@@ -1793,24 +1757,24 @@
       <c r="F9" s="55"/>
       <c r="G9" s="39"/>
       <c r="H9" s="40"/>
-      <c r="I9" s="120"/>
-      <c r="J9" s="116"/>
-      <c r="K9" s="102"/>
+      <c r="I9" s="116"/>
+      <c r="J9" s="112"/>
+      <c r="K9" s="98"/>
       <c r="L9" s="95"/>
-      <c r="M9" s="103"/>
+      <c r="M9" s="99"/>
       <c r="N9" s="91"/>
       <c r="O9" s="43"/>
       <c r="P9" s="44"/>
       <c r="Q9" s="45"/>
-      <c r="R9" s="124"/>
+      <c r="R9" s="120"/>
       <c r="S9" s="46"/>
       <c r="T9" s="47"/>
       <c r="U9" s="46"/>
       <c r="V9" s="46"/>
-      <c r="W9" s="129"/>
-      <c r="X9" s="140"/>
-    </row>
-    <row r="10" spans="1:53" s="53" customFormat="1" ht="84.6" customHeight="1">
+      <c r="W9" s="125"/>
+      <c r="X9" s="131"/>
+    </row>
+    <row r="10" spans="1:53" s="53" customFormat="1" ht="84.5" customHeight="1">
       <c r="A10" s="56"/>
       <c r="B10" s="89"/>
       <c r="C10" s="49"/>
@@ -1819,8 +1783,8 @@
       <c r="F10" s="55"/>
       <c r="G10" s="39"/>
       <c r="H10" s="40"/>
-      <c r="I10" s="120"/>
-      <c r="J10" s="116"/>
+      <c r="I10" s="116"/>
+      <c r="J10" s="112"/>
       <c r="K10" s="90"/>
       <c r="L10" s="51"/>
       <c r="M10" s="42"/>
@@ -1828,15 +1792,15 @@
       <c r="O10" s="43"/>
       <c r="P10" s="44"/>
       <c r="Q10" s="45"/>
-      <c r="R10" s="125"/>
+      <c r="R10" s="121"/>
       <c r="S10" s="46"/>
       <c r="T10" s="47"/>
       <c r="U10" s="46"/>
       <c r="V10" s="46"/>
-      <c r="W10" s="130" t="s">
+      <c r="W10" s="126" t="s">
         <v>20</v>
       </c>
-      <c r="X10" s="140"/>
+      <c r="X10" s="131"/>
       <c r="Y10" s="52"/>
       <c r="Z10" s="52"/>
       <c r="AA10" s="52"/>
@@ -1867,7 +1831,7 @@
       <c r="AZ10" s="52"/>
       <c r="BA10" s="52"/>
     </row>
-    <row r="11" spans="1:53" s="35" customFormat="1" ht="84.6" customHeight="1">
+    <row r="11" spans="1:53" s="35" customFormat="1" ht="84.5" customHeight="1">
       <c r="A11" s="48"/>
       <c r="B11" s="89"/>
       <c r="C11" s="54"/>
@@ -1876,8 +1840,8 @@
       <c r="F11" s="55"/>
       <c r="G11" s="39"/>
       <c r="H11" s="40"/>
-      <c r="I11" s="120"/>
-      <c r="J11" s="116"/>
+      <c r="I11" s="116"/>
+      <c r="J11" s="112"/>
       <c r="K11" s="90"/>
       <c r="L11" s="51"/>
       <c r="M11" s="42"/>
@@ -1885,15 +1849,15 @@
       <c r="O11" s="43"/>
       <c r="P11" s="44"/>
       <c r="Q11" s="45"/>
-      <c r="R11" s="124"/>
+      <c r="R11" s="120"/>
       <c r="S11" s="46"/>
       <c r="T11" s="47"/>
       <c r="U11" s="46"/>
       <c r="V11" s="46"/>
-      <c r="W11" s="129"/>
-      <c r="X11" s="140"/>
-    </row>
-    <row r="12" spans="1:53" s="53" customFormat="1" ht="84.6" customHeight="1">
+      <c r="W11" s="125"/>
+      <c r="X11" s="131"/>
+    </row>
+    <row r="12" spans="1:53" s="53" customFormat="1" ht="84.5" customHeight="1">
       <c r="A12" s="56"/>
       <c r="B12" s="88"/>
       <c r="C12" s="37"/>
@@ -1902,8 +1866,8 @@
       <c r="F12" s="55"/>
       <c r="G12" s="39"/>
       <c r="H12" s="40"/>
-      <c r="I12" s="120"/>
-      <c r="J12" s="116"/>
+      <c r="I12" s="116"/>
+      <c r="J12" s="112"/>
       <c r="K12" s="90"/>
       <c r="L12" s="41"/>
       <c r="M12" s="42"/>
@@ -1911,13 +1875,13 @@
       <c r="O12" s="43"/>
       <c r="P12" s="44"/>
       <c r="Q12" s="45"/>
-      <c r="R12" s="125"/>
+      <c r="R12" s="121"/>
       <c r="S12" s="46"/>
       <c r="T12" s="47"/>
       <c r="U12" s="46"/>
       <c r="V12" s="46"/>
-      <c r="W12" s="130"/>
-      <c r="X12" s="140"/>
+      <c r="W12" s="126"/>
+      <c r="X12" s="131"/>
       <c r="Y12" s="52"/>
       <c r="Z12" s="52"/>
       <c r="AA12" s="52"/>
@@ -1948,7 +1912,7 @@
       <c r="AZ12" s="52"/>
       <c r="BA12" s="52"/>
     </row>
-    <row r="13" spans="1:53" s="64" customFormat="1" ht="84.6" customHeight="1" thickBot="1">
+    <row r="13" spans="1:53" s="64" customFormat="1" ht="84.5" customHeight="1" thickBot="1">
       <c r="A13" s="57"/>
       <c r="B13" s="57"/>
       <c r="C13" s="58"/>
@@ -1957,25 +1921,27 @@
       <c r="F13" s="55"/>
       <c r="G13" s="61"/>
       <c r="H13" s="40"/>
-      <c r="I13" s="119"/>
-      <c r="J13" s="133"/>
-      <c r="K13" s="134"/>
-      <c r="L13" s="109"/>
-      <c r="M13" s="110"/>
+      <c r="I13" s="115"/>
+      <c r="J13" s="129"/>
+      <c r="K13" s="130"/>
+      <c r="L13" s="105"/>
+      <c r="M13" s="106"/>
       <c r="N13" s="91"/>
       <c r="O13" s="62"/>
       <c r="P13" s="44"/>
       <c r="Q13" s="63"/>
-      <c r="R13" s="126"/>
+      <c r="R13" s="122"/>
       <c r="S13" s="46"/>
       <c r="T13" s="47"/>
       <c r="U13" s="46"/>
       <c r="V13" s="46"/>
-      <c r="W13" s="131"/>
-      <c r="X13" s="141"/>
+      <c r="W13" s="127"/>
+      <c r="X13" s="132"/>
     </row>
     <row r="14" spans="1:53" s="53" customFormat="1" ht="36" customHeight="1" thickBot="1">
-      <c r="A14" s="65"/>
+      <c r="A14" s="65" t="s">
+        <v>35</v>
+      </c>
       <c r="B14" s="66"/>
       <c r="C14" s="67"/>
       <c r="D14" s="68"/>
@@ -1986,14 +1952,14 @@
         <f>SUM(H9:H13)</f>
         <v>0</v>
       </c>
-      <c r="I14" s="117"/>
-      <c r="J14" s="117"/>
-      <c r="K14" s="118">
+      <c r="I14" s="113"/>
+      <c r="J14" s="113"/>
+      <c r="K14" s="114">
         <f>SUM(K9:K13)</f>
         <v>0</v>
       </c>
-      <c r="L14" s="111"/>
-      <c r="M14" s="112" t="s">
+      <c r="L14" s="107"/>
+      <c r="M14" s="108" t="s">
         <v>21</v>
       </c>
       <c r="N14" s="94">
@@ -2040,23 +2006,25 @@
       <c r="AZ14" s="52"/>
       <c r="BA14" s="52"/>
     </row>
-    <row r="15" spans="1:53" s="53" customFormat="1" ht="31.5" customHeight="1">
-      <c r="A15" s="70"/>
-      <c r="B15" s="70"/>
-      <c r="C15" s="74"/>
-      <c r="D15" s="75"/>
-      <c r="E15" s="70"/>
-      <c r="F15" s="75"/>
-      <c r="G15" s="98"/>
-      <c r="H15" s="98"/>
-      <c r="I15" s="99"/>
-      <c r="J15" s="99"/>
-      <c r="K15" s="108"/>
-      <c r="L15" s="111"/>
-      <c r="M15" s="115" t="s">
+    <row r="15" spans="1:53" s="53" customFormat="1" ht="40">
+      <c r="A15" s="133"/>
+      <c r="B15" s="133" t="s">
+        <v>36</v>
+      </c>
+      <c r="C15" s="133"/>
+      <c r="D15" s="133"/>
+      <c r="E15" s="133"/>
+      <c r="F15" s="133"/>
+      <c r="G15" s="133"/>
+      <c r="H15" s="134"/>
+      <c r="I15" s="135"/>
+      <c r="J15" s="135"/>
+      <c r="K15" s="104"/>
+      <c r="L15" s="107"/>
+      <c r="M15" s="111" t="s">
         <v>31</v>
       </c>
-      <c r="N15" s="104">
+      <c r="N15" s="100">
         <v>6</v>
       </c>
       <c r="O15" s="78"/>
@@ -2099,21 +2067,17 @@
       <c r="AZ15" s="52"/>
       <c r="BA15" s="52"/>
     </row>
-    <row r="16" spans="1:53" ht="30" customHeight="1">
-      <c r="G16" s="100"/>
-      <c r="H16" s="100"/>
-      <c r="I16" s="101"/>
-      <c r="J16" s="101"/>
-      <c r="L16" s="113"/>
-      <c r="M16" s="114" t="s">
+    <row r="16" spans="1:53" ht="26">
+      <c r="L16" s="109"/>
+      <c r="M16" s="110" t="s">
         <v>27</v>
       </c>
-      <c r="N16" s="105">
+      <c r="N16" s="101">
         <f>N14*N15</f>
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:21" ht="17.399999999999999" customHeight="1">
+    <row r="17" spans="1:21">
       <c r="C17" s="70"/>
       <c r="D17" s="70"/>
       <c r="F17" s="70"/>
@@ -2127,18 +2091,18 @@
       <c r="T17" s="70"/>
       <c r="U17" s="70"/>
     </row>
-    <row r="19" spans="1:21" s="107" customFormat="1" ht="38.25" customHeight="1">
-      <c r="A19" s="127"/>
-      <c r="D19" s="127"/>
-      <c r="H19" s="127"/>
-    </row>
-    <row r="20" spans="1:21" s="107" customFormat="1" ht="38.25" customHeight="1">
-      <c r="B20" s="128"/>
-      <c r="E20" s="128"/>
-      <c r="I20" s="128"/>
-      <c r="J20" s="128"/>
-    </row>
-    <row r="21" spans="1:21" ht="17.399999999999999" customHeight="1">
+    <row r="19" spans="1:21" s="103" customFormat="1" ht="18" customHeight="1">
+      <c r="A19" s="123"/>
+      <c r="D19" s="123"/>
+      <c r="H19" s="123"/>
+    </row>
+    <row r="20" spans="1:21" s="103" customFormat="1" ht="18" customHeight="1">
+      <c r="B20" s="124"/>
+      <c r="E20" s="124"/>
+      <c r="I20" s="124"/>
+      <c r="J20" s="124"/>
+    </row>
+    <row r="21" spans="1:21" ht="18" customHeight="1">
       <c r="C21" s="70"/>
       <c r="D21" s="70"/>
       <c r="F21" s="70"/>
@@ -2152,7 +2116,7 @@
       <c r="T21" s="70"/>
       <c r="U21" s="70"/>
     </row>
-    <row r="22" spans="1:21" ht="17.399999999999999" customHeight="1">
+    <row r="22" spans="1:21" ht="18" customHeight="1">
       <c r="C22" s="70"/>
       <c r="D22" s="70"/>
       <c r="F22" s="70"/>
@@ -2166,7 +2130,7 @@
       <c r="T22" s="70"/>
       <c r="U22" s="70"/>
     </row>
-    <row r="23" spans="1:21" ht="17.399999999999999" customHeight="1">
+    <row r="23" spans="1:21">
       <c r="C23" s="70"/>
       <c r="D23" s="70"/>
       <c r="F23" s="70"/>
@@ -2180,7 +2144,7 @@
       <c r="T23" s="70"/>
       <c r="U23" s="70"/>
     </row>
-    <row r="24" spans="1:21" ht="17.399999999999999" customHeight="1">
+    <row r="24" spans="1:21">
       <c r="C24" s="70"/>
       <c r="D24" s="70"/>
       <c r="F24" s="70"/>
@@ -2194,7 +2158,7 @@
       <c r="T24" s="70"/>
       <c r="U24" s="70"/>
     </row>
-    <row r="25" spans="1:21" ht="17.399999999999999" customHeight="1">
+    <row r="25" spans="1:21">
       <c r="C25" s="70"/>
       <c r="D25" s="70"/>
       <c r="F25" s="70"/>
@@ -2208,7 +2172,7 @@
       <c r="T25" s="70"/>
       <c r="U25" s="70"/>
     </row>
-    <row r="26" spans="1:21" ht="17.399999999999999" customHeight="1">
+    <row r="26" spans="1:21">
       <c r="C26" s="70"/>
       <c r="D26" s="70"/>
       <c r="F26" s="70"/>
@@ -2222,7 +2186,7 @@
       <c r="T26" s="70"/>
       <c r="U26" s="70"/>
     </row>
-    <row r="27" spans="1:21" ht="17.399999999999999" customHeight="1">
+    <row r="27" spans="1:21" ht="17" customHeight="1">
       <c r="C27" s="70"/>
       <c r="D27" s="70"/>
       <c r="F27" s="70"/>
@@ -2236,7 +2200,7 @@
       <c r="T27" s="70"/>
       <c r="U27" s="70"/>
     </row>
-    <row r="28" spans="1:21" ht="17.399999999999999" customHeight="1">
+    <row r="28" spans="1:21" ht="17.5" customHeight="1">
       <c r="C28" s="70"/>
       <c r="D28" s="70"/>
       <c r="F28" s="70"/>
@@ -2250,7 +2214,7 @@
       <c r="T28" s="70"/>
       <c r="U28" s="70"/>
     </row>
-    <row r="29" spans="1:21" ht="17.399999999999999" customHeight="1">
+    <row r="29" spans="1:21" ht="17.5" customHeight="1">
       <c r="C29" s="70"/>
       <c r="D29" s="70"/>
       <c r="F29" s="70"/>
@@ -2264,7 +2228,7 @@
       <c r="T29" s="70"/>
       <c r="U29" s="70"/>
     </row>
-    <row r="30" spans="1:21" ht="17.399999999999999" customHeight="1">
+    <row r="30" spans="1:21" ht="17.5" customHeight="1">
       <c r="C30" s="70"/>
       <c r="D30" s="70"/>
       <c r="F30" s="70"/>
@@ -2278,7 +2242,7 @@
       <c r="T30" s="70"/>
       <c r="U30" s="70"/>
     </row>
-    <row r="31" spans="1:21" ht="17.399999999999999" customHeight="1">
+    <row r="31" spans="1:21" ht="17.5" customHeight="1">
       <c r="C31" s="70"/>
       <c r="D31" s="70"/>
       <c r="F31" s="70"/>
@@ -2292,7 +2256,7 @@
       <c r="T31" s="70"/>
       <c r="U31" s="70"/>
     </row>
-    <row r="32" spans="1:21" ht="17.399999999999999" customHeight="1">
+    <row r="32" spans="1:21" ht="17.5" customHeight="1">
       <c r="C32" s="70"/>
       <c r="D32" s="70"/>
       <c r="F32" s="70"/>
@@ -2306,336 +2270,336 @@
       <c r="T32" s="70"/>
       <c r="U32" s="70"/>
     </row>
-    <row r="33" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="34" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="35" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="36" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="37" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="38" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="39" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="40" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="41" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="42" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="43" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="44" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="45" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="46" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="47" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="48" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="49" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="50" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="51" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="52" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="53" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="54" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="55" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="56" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="57" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="58" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="59" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="60" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="61" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="62" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="63" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="64" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="65" s="70" customFormat="1" ht="34.950000000000003" customHeight="1"/>
-    <row r="66" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="67" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="68" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="69" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="70" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="71" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="72" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="73" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="74" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="75" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="76" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="77" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="78" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="79" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="80" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="81" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="82" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="83" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="84" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="85" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="86" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="87" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="88" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="89" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="90" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="91" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="92" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="93" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="94" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="95" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="96" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="97" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="98" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="99" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="100" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="101" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="102" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="103" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="104" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="105" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="106" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="107" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="108" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="109" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="110" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="111" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="112" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="113" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="114" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="115" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="116" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="117" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="118" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="119" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="120" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="121" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="122" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="123" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="124" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="125" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="126" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="127" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="128" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="129" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="130" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="131" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="132" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="133" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="134" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="135" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="136" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="137" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="138" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="139" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="140" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="141" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="142" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="143" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="144" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="145" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="146" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="147" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="148" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="149" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="150" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="151" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="152" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="153" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="154" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="155" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="156" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="157" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="158" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="159" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="160" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="161" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="162" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="163" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="164" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="165" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="166" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="167" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="168" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="169" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="170" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="171" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="172" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="173" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="174" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="175" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="176" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="177" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="178" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="179" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="180" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="181" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="182" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="183" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="184" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="185" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="186" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="187" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="188" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="189" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="190" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="191" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="192" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="193" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="194" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="195" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="196" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="197" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="198" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="199" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="200" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="201" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="202" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="203" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="204" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="205" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="206" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="207" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="208" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="209" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="210" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="211" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="212" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="213" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="214" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="215" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="216" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="217" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="218" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="219" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="220" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="221" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="222" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="223" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="224" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="225" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="226" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="227" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="228" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="229" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="230" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="231" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="232" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="233" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="234" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="235" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="236" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="237" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="238" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="239" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="240" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="241" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="242" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="243" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="244" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="245" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="246" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="247" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="248" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="249" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="250" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="251" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="252" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="253" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="254" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="255" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="256" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="257" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="258" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="259" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="260" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="261" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="262" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="263" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="264" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="265" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="266" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="267" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="268" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="269" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="270" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="271" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="272" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="273" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="274" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="275" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="276" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="277" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="278" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="279" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="280" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="281" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="282" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="283" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="284" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="285" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="286" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="287" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="288" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="289" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="290" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="291" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="292" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="293" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="294" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="295" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="296" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="297" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="298" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="299" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="300" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="301" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="302" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="303" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="304" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="305" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="306" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="307" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="308" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="309" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="310" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="311" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="312" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="313" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="314" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="315" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="316" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="317" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="318" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="319" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="320" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="321" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="322" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="323" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="324" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="325" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="326" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="327" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="328" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="329" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="330" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="331" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="332" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="333" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="334" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="335" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="336" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="337" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="338" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="339" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="340" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="341" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="342" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="343" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="344" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="345" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="346" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="347" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="348" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="349" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="350" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="351" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="352" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="353" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="354" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="355" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="356" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="357" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="358" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="359" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="360" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="361" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
-    <row r="362" s="70" customFormat="1" ht="17.399999999999999" customHeight="1"/>
+    <row r="33" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="34" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="35" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="36" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="37" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="38" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="39" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="40" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="41" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="42" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="43" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="44" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="45" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="46" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="47" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="48" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="49" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="50" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="51" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="52" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="53" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="54" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="55" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="56" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="57" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="58" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="59" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="60" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="61" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="62" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="63" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="64" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="65" s="70" customFormat="1" ht="18" customHeight="1"/>
+    <row r="66" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="67" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="68" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="69" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="70" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="71" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="72" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="73" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="74" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="75" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="76" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="77" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="78" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="79" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="80" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="81" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="82" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="83" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="84" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="85" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="86" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="87" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="88" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="89" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="90" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="91" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="92" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="93" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="94" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="95" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="96" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="97" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="98" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="99" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="100" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="101" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="102" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="103" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="104" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="105" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="106" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="107" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="108" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="109" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="110" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="111" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="112" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="113" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="114" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="115" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="116" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="117" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="118" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="119" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="120" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="121" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="122" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="123" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="124" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="125" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="126" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="127" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="128" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="129" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="130" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="131" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="132" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="133" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="134" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="135" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="136" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="137" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="138" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="139" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="140" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="141" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="142" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="143" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="144" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="145" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="146" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="147" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="148" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="149" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="150" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="151" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="152" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="153" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="154" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="155" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="156" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="157" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="158" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="159" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="160" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="161" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="162" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="163" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="164" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="165" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="166" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="167" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="168" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="169" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="170" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="171" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="172" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="173" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="174" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="175" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="176" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="177" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="178" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="179" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="180" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="181" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="182" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="183" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="184" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="185" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="186" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="187" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="188" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="189" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="190" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="191" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="192" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="193" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="194" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="195" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="196" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="197" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="198" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="199" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="200" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="201" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="202" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="203" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="204" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="205" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="206" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="207" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="208" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="209" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="210" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="211" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="212" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="213" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="214" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="215" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="216" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="217" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="218" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="219" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="220" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="221" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="222" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="223" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="224" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="225" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="226" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="227" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="228" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="229" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="230" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="231" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="232" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="233" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="234" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="235" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="236" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="237" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="238" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="239" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="240" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="241" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="242" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="243" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="244" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="245" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="246" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="247" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="248" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="249" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="250" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="251" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="252" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="253" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="254" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="255" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="256" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="257" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="258" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="259" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="260" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="261" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="262" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="263" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="264" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="265" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="266" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="267" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="268" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="269" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="270" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="271" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="272" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="273" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="274" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="275" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="276" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="277" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="278" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="279" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="280" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="281" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="282" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="283" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="284" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="285" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="286" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="287" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="288" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="289" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="290" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="291" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="292" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="293" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="294" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="295" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="296" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="297" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="298" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="299" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="300" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="301" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="302" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="303" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="304" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="305" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="306" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="307" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="308" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="309" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="310" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="311" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="312" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="313" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="314" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="315" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="316" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="317" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="318" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="319" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="320" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="321" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="322" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="323" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="324" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="325" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="326" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="327" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="328" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="329" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="330" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="331" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="332" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="333" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="334" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="335" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="336" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="337" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="338" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="339" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="340" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="341" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="342" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="343" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="344" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="345" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="346" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="347" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="348" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="349" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="350" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="351" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="352" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="353" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="354" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="355" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="356" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="357" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="358" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="359" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="360" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="361" s="70" customFormat="1" ht="17.5" customHeight="1"/>
+    <row r="362" s="70" customFormat="1" ht="17.5" customHeight="1"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="C1:F1"/>
@@ -2645,6 +2609,5 @@
   <pageMargins left="0.14000000000000001" right="0.12" top="0.36" bottom="0.36" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="40" fitToHeight="0" orientation="landscape" verticalDpi="180" r:id="rId1"/>
   <headerFooter alignWithMargins="0"/>
-  <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>